<commit_message>
Update crew schedule spreadsheet 2026-05-10
</commit_message>
<xml_diff>
--- a/data/crew-schedule.xlsx
+++ b/data/crew-schedule.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="May 04" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="May 11" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1375,4 +1376,829 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Crew Schedule - Week of May 11, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Arlington: Cycle active: 2026-04-27 - 2026-05-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>NEW: Ridglea Court Apartments - $8,414</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Property</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Budget Hrs</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Crew</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Capp Smith Park</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>31-cycle. VERIFY on Watauga Park Schedule PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Central Fire Station</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>31-cycle, adjacent</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Hillview Park</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>31-cycle, adjacent</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Public Works Facility</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>31-cycle, 1 min north</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Animal Service Center</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>31-cycle, last Watauga stop</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Leo at Bethel</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Full day, single property</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Miller Milling</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>5.32</v>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>Saginaw, weekly</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Crowley Creekside HOA</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>42</v>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>Moved from Fri per Evelin 4/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Dakota Apartments</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>5.72</v>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>Weekly, fixed on Tue</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>BISD Park</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>31-cycle. VERIFY on park schedule PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Foster Village Park</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>31-cycle, largest first</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Municipal Complex</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>31-cycle, adjacent</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Virgil Anthony Park</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>31-cycle, last Watauga stop</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>Five Oaks Crossing</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>Mansfield, first heading south</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>Craft Residence</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>RESIDENTIAL - Thu/Fri only</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>Carol Katz Residence</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>RESIDENTIAL - Thu/Fri only</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>Nick Workman Residence</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>RESIDENTIAL - Thu/Fri only</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>BASIS Benbrook</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>Morning stop, Benbrook</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>University Christian Church</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>AFTERNOON ONLY - do after lunch</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>Watauga Community Center</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F25" s="11" t="inlineStr">
+        <is>
+          <t>31-cycle. Last Watauga stop (done by Thu)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Bear Creek HOA</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Cresson, first heading south</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Parcel B</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Continue south</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Tom Brown Residence</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>RESIDENTIAL - Thu/Fri only</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Richard Watters Residence</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>RESIDENTIAL - Thu/Fri only</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Creekside Field Mow</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Bi-weekly (Opp 3146)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>Weekly Hours Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>Gustavo (hrs/person)</t>
+        </is>
+      </c>
+      <c r="D33" s="15" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="E33" s="16" t="inlineStr">
+        <is>
+          <t>OT: 0.0 hrs</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>Jorge (hrs/person)</t>
+        </is>
+      </c>
+      <c r="D34" s="15" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="E34" s="16" t="inlineStr">
+        <is>
+          <t>OT: 0.0 hrs</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="17" t="inlineStr">
+        <is>
+          <t>Generated 2026-05-10 02:50 PM</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A32:F32"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update crew schedule spreadsheet 2026-05-17
</commit_message>
<xml_diff>
--- a/data/crew-schedule.xlsx
+++ b/data/crew-schedule.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="May 04" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="May 11" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="May 18" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,6 +66,12 @@
       <name val="Arial"/>
       <color rgb="00888888"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00006600"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="9">
@@ -135,7 +142,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -166,6 +173,7 @@
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2201,4 +2209,849 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Crew Schedule - Week of May 18, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="18" t="inlineStr">
+        <is>
+          <t>Arlington: Gap week — Daniel/Saul available for overflow</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Property</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Budget Hrs</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Crew</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Capp Smith Park</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>31-cycle. VERIFY on Watauga Park Schedule PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Central Fire Station</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>31-cycle, adjacent</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Hillview Park</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>31-cycle, adjacent</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Public Works Facility</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>31-cycle, 1 min north</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Animal Service Center</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>31-cycle, last Watauga stop</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Leo at Bethel</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Full day, single property</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Miller Milling</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>5.32</v>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Saginaw, weekly</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Crowley Creekside HOA</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>42</v>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>Moved from Fri per Evelin 4/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Dakota Apartments</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>5.72</v>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>Weekly, fixed on Tue</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>BISD Park</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>31-cycle. VERIFY on park schedule PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Whites Branch Creek Trail</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>21-cycle. VERIFY on park schedule PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Foster Village Park</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>31-cycle, largest first</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Municipal Complex</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>31-cycle, adjacent</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Virgil Anthony Park</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>31-cycle, last Watauga stop</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>Five Oaks Crossing</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>Mansfield, first heading south</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>Craft Residence</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>RESIDENTIAL - Thu/Fri only</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>Carol Katz Residence</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>RESIDENTIAL - Thu/Fri only</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>Nick Workman Residence</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>RESIDENTIAL - Thu/Fri only</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>BASIS Benbrook</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>Morning stop, Benbrook</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>University Christian Church</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>AFTERNOON ONLY - do after lunch</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>Watauga Community Center</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F25" s="11" t="inlineStr">
+        <is>
+          <t>31-cycle. Last Watauga stop (done by Thu)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Bear Creek HOA</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Cresson, first heading south</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Parcel B</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Continue south</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Tom Brown Residence</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>RESIDENTIAL - Thu/Fri only</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Richard Watters Residence</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>RESIDENTIAL - Thu/Fri only</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Hampton Manor</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="n">
+        <v>7.34</v>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Bi-weekly (24/yr)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>Weekly Hours Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>Gustavo (hrs/person)</t>
+        </is>
+      </c>
+      <c r="D33" s="15" t="n">
+        <v>31.9</v>
+      </c>
+      <c r="E33" s="16" t="inlineStr">
+        <is>
+          <t>OT: 0.0 hrs</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>Jorge (hrs/person)</t>
+        </is>
+      </c>
+      <c r="D34" s="15" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="E34" s="16" t="inlineStr">
+        <is>
+          <t>OT: 0.0 hrs</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="17" t="inlineStr">
+        <is>
+          <t>Generated 2026-05-17 02:53 PM</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A32:F32"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update crew schedule spreadsheet 2026-05-24
</commit_message>
<xml_diff>
--- a/data/crew-schedule.xlsx
+++ b/data/crew-schedule.xlsx
@@ -10,6 +10,7 @@
     <sheet name="May 04" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="May 11" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="May 18" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="May 25" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3054,4 +3055,821 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Crew Schedule - Week of May 25, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="18" t="inlineStr">
+        <is>
+          <t>Arlington: Gap week — Daniel/Saul available for overflow</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Property</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Budget Hrs</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Crew</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Capp Smith Park</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>31-cycle. VERIFY on Watauga Park Schedule PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Central Fire Station</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>31-cycle, adjacent</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Hillview Park</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>31-cycle, adjacent</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Public Works Facility</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>31-cycle, 1 min north</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Animal Service Center</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>31-cycle, last Watauga stop</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Leo at Bethel</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Full day, single property</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Miller Milling</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>5.32</v>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Saginaw, weekly</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Crowley Creekside HOA</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>42</v>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>Moved from Fri per Evelin 4/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Dakota Apartments</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>5.72</v>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>Weekly, fixed on Tue</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>BISD Park</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>31-cycle. VERIFY on park schedule PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Foster Village Park</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>31-cycle, largest first</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Municipal Complex</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>31-cycle, adjacent</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Virgil Anthony Park</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>31-cycle, last Watauga stop</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Five Oaks Crossing</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>Mansfield, first heading south</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>Craft Residence</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>RESIDENTIAL - Thu/Fri only</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>Carol Katz Residence</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>RESIDENTIAL - Thu/Fri only</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>Nick Workman Residence</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>RESIDENTIAL - Thu/Fri only</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>BASIS Benbrook</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>Morning stop, Benbrook</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>University Christian Church</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>AFTERNOON ONLY - do after lunch</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>Watauga Community Center</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>31-cycle. Last Watauga stop (done by Thu)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Bear Creek HOA</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Cresson, first heading south</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Parcel B</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Continue south</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Tom Brown Residence</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>RESIDENTIAL - Thu/Fri only</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Richard Watters Residence</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>RESIDENTIAL - Thu/Fri only</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Creekside Field Mow</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Bi-weekly (Opp 3146)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>Weekly Hours Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>Gustavo (hrs/person)</t>
+        </is>
+      </c>
+      <c r="D32" s="15" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="E32" s="16" t="inlineStr">
+        <is>
+          <t>OT: 0.0 hrs</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>Jorge (hrs/person)</t>
+        </is>
+      </c>
+      <c r="D33" s="15" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="E33" s="16" t="inlineStr">
+        <is>
+          <t>OT: 0.0 hrs</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="17" t="inlineStr">
+        <is>
+          <t>Generated 2026-05-24 02:31 PM</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update crew schedule spreadsheet 2026-05-31
</commit_message>
<xml_diff>
--- a/data/crew-schedule.xlsx
+++ b/data/crew-schedule.xlsx
@@ -11,6 +11,7 @@
     <sheet name="May 11" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="May 18" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="May 25" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Jun 01" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3872,4 +3873,849 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Crew Schedule - Week of June 01, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="18" t="inlineStr">
+        <is>
+          <t>Arlington: Gap week — Daniel/Saul available for overflow</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Property</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Budget Hrs</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Crew</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Capp Smith Park</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>31-cycle. VERIFY on Watauga Park Schedule PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Central Fire Station</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>31-cycle, adjacent</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Hillview Park</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>31-cycle, adjacent</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Public Works Facility</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>31-cycle, 1 min north</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Animal Service Center</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>31-cycle, last Watauga stop</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Leo at Bethel</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Full day, single property</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Miller Milling</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>5.32</v>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Saginaw, weekly</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Crowley Creekside HOA</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>42</v>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>Moved from Fri per Evelin 4/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Dakota Apartments</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>5.72</v>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>Weekly, fixed on Tue</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>BISD Park</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>31-cycle. VERIFY on park schedule PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Whites Branch Creek Trail</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>21-cycle. VERIFY on park schedule PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Foster Village Park</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>31-cycle, largest first</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Municipal Complex</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>31-cycle, adjacent</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Virgil Anthony Park</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>31-cycle, last Watauga stop</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>Five Oaks Crossing</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>Mansfield, first heading south</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>Craft Residence</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>RESIDENTIAL - Thu/Fri only</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>Carol Katz Residence</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>RESIDENTIAL - Thu/Fri only</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>Nick Workman Residence</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>RESIDENTIAL - Thu/Fri only</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>BASIS Benbrook</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>Morning stop, Benbrook</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>University Christian Church</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>AFTERNOON ONLY - do after lunch</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>Watauga Community Center</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F25" s="11" t="inlineStr">
+        <is>
+          <t>31-cycle. Last Watauga stop (done by Thu)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Bear Creek HOA</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Cresson, first heading south</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Parcel B</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Continue south</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Tom Brown Residence</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>RESIDENTIAL - Thu/Fri only</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Richard Watters Residence</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>RESIDENTIAL - Thu/Fri only</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Hampton Manor</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="n">
+        <v>7.34</v>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Bi-weekly (24/yr)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>Weekly Hours Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>Gustavo (hrs/person)</t>
+        </is>
+      </c>
+      <c r="D33" s="15" t="n">
+        <v>31.9</v>
+      </c>
+      <c r="E33" s="16" t="inlineStr">
+        <is>
+          <t>OT: 0.0 hrs</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>Jorge (hrs/person)</t>
+        </is>
+      </c>
+      <c r="D34" s="15" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="E34" s="16" t="inlineStr">
+        <is>
+          <t>OT: 0.0 hrs</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="17" t="inlineStr">
+        <is>
+          <t>Generated 2026-05-31 03:16 PM</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A32:F32"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update crew schedule spreadsheet 2026-06-07
</commit_message>
<xml_diff>
--- a/data/crew-schedule.xlsx
+++ b/data/crew-schedule.xlsx
@@ -12,6 +12,7 @@
     <sheet name="May 18" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="May 25" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Jun 01" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Jun 08" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4718,4 +4719,821 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Crew Schedule - Week of June 08, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="18" t="inlineStr">
+        <is>
+          <t>Arlington: Gap week — Daniel/Saul available for overflow</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Property</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Budget Hrs</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Crew</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Capp Smith Park</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>31-cycle. VERIFY on Watauga Park Schedule PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Central Fire Station</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>31-cycle, adjacent</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Hillview Park</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>31-cycle, adjacent</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Public Works Facility</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>31-cycle, 1 min north</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Animal Service Center</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>31-cycle, last Watauga stop</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Leo at Bethel</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Full day, single property</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Miller Milling</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>5.32</v>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Saginaw, weekly</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Crowley Creekside HOA</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>42</v>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>Moved from Fri per Evelin 4/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Dakota Apartments</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>5.72</v>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>Weekly, fixed on Tue</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>BISD Park</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>31-cycle. VERIFY on park schedule PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Foster Village Park</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>31-cycle, largest first</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Municipal Complex</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>31-cycle, adjacent</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Virgil Anthony Park</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>31-cycle, last Watauga stop</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Five Oaks Crossing</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>Mansfield, first heading south</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>Craft Residence</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>RESIDENTIAL - Thu/Fri only</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>Carol Katz Residence</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>RESIDENTIAL - Thu/Fri only</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>Nick Workman Residence</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>RESIDENTIAL - Thu/Fri only</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>BASIS Benbrook</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>Morning stop, Benbrook</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>University Christian Church</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>AFTERNOON ONLY - do after lunch</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>Watauga Community Center</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>31-cycle. Last Watauga stop (done by Thu)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Bear Creek HOA</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Cresson, first heading south</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Parcel B</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Continue south</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Tom Brown Residence</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>RESIDENTIAL - Thu/Fri only</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Richard Watters Residence</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>RESIDENTIAL - Thu/Fri only</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Creekside Field Mow</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Jorge</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Bi-weekly (Opp 3146)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>Weekly Hours Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>Gustavo (hrs/person)</t>
+        </is>
+      </c>
+      <c r="D32" s="15" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="E32" s="16" t="inlineStr">
+        <is>
+          <t>OT: 0.0 hrs</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>Jorge (hrs/person)</t>
+        </is>
+      </c>
+      <c r="D33" s="15" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="E33" s="16" t="inlineStr">
+        <is>
+          <t>OT: 0.0 hrs</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="17" t="inlineStr">
+        <is>
+          <t>Generated 2026-06-07 03:22 PM</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>